<commit_message>
Amber : P : RP : RheinWedDe : add ferienwohnung sheet in wiesbaden.xlsx
</commit_message>
<xml_diff>
--- a/P(Path)/RP(Rhine-Path)/RheinWegDE/Wiesbaden.xlsx
+++ b/P(Path)/RP(Rhine-Path)/RheinWegDE/Wiesbaden.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="restaurant" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kino" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="taxi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ferienwohnung" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -46621,4 +46622,1570 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" style="7" min="1" max="1"/>
+    <col width="34.66" customWidth="1" style="7" min="2" max="2"/>
+    <col width="22" customWidth="1" style="7" min="3" max="3"/>
+    <col width="36" customWidth="1" style="7" min="4" max="4"/>
+    <col width="12" customWidth="1" style="7" min="5" max="5"/>
+    <col width="10" customWidth="1" style="7" min="6" max="6"/>
+    <col width="28" customWidth="1" style="7" min="7" max="7"/>
+    <col width="28" customWidth="1" style="7" min="8" max="8"/>
+    <col width="18" customWidth="1" style="7" min="9" max="9"/>
+    <col width="16" customWidth="1" style="7" min="10" max="10"/>
+    <col width="16" customWidth="1" style="7" min="11" max="11"/>
+    <col width="16" customWidth="1" style="7" min="12" max="12"/>
+    <col width="32" customWidth="1" style="7" min="13" max="13"/>
+    <col width="32" customWidth="1" style="7" min="14" max="14"/>
+    <col width="40" customWidth="1" style="7" min="15" max="15"/>
+    <col width="42" customWidth="1" style="7" min="16" max="16"/>
+    <col width="26" customWidth="1" style="7" min="17" max="17"/>
+    <col width="9" customWidth="1" style="7" min="18" max="18"/>
+    <col width="10" customWidth="1" style="7" min="19" max="19"/>
+    <col width="11" customWidth="1" style="7" min="20" max="20"/>
+    <col width="16" customWidth="1" style="7" min="21" max="21"/>
+    <col width="45" customWidth="1" style="7" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1" s="7">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>🏠  Ferienwohnung – Wiesbaden  ·  19 Companies  ·  Source: GelbeSeiten</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" s="7">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
+        <is>
+          <t>Business Description</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Province</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>ZIP Code</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="H2" s="11" t="inlineStr">
+        <is>
+          <t>Street</t>
+        </is>
+      </c>
+      <c r="I2" s="11" t="inlineStr">
+        <is>
+          <t>Contact Person</t>
+        </is>
+      </c>
+      <c r="J2" s="11" t="inlineStr">
+        <is>
+          <t>Telephone 1</t>
+        </is>
+      </c>
+      <c r="K2" s="11" t="inlineStr">
+        <is>
+          <t>Telephone 2</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
+        <is>
+          <t>Telephone 3</t>
+        </is>
+      </c>
+      <c r="M2" s="11" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="N2" s="11" t="inlineStr">
+        <is>
+          <t>Email 2</t>
+        </is>
+      </c>
+      <c r="O2" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="P2" s="11" t="inlineStr">
+        <is>
+          <t>Social Media</t>
+        </is>
+      </c>
+      <c r="Q2" s="11" t="inlineStr">
+        <is>
+          <t>Opening Hours</t>
+        </is>
+      </c>
+      <c r="R2" s="11" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="S2" s="11" t="inlineStr">
+        <is>
+          <t># Reviews</t>
+        </is>
+      </c>
+      <c r="T2" s="11" t="inlineStr">
+        <is>
+          <t>Distance</t>
+        </is>
+      </c>
+      <c r="U2" s="11" t="inlineStr">
+        <is>
+          <t>Badge / Partner</t>
+        </is>
+      </c>
+      <c r="V2" s="11" t="inlineStr">
+        <is>
+          <t>GelbeSeiten URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>DERTOUR Reisebüro</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Fernreisen, Kreuzfahrten, Rundreisen, Ferienwohnung, Mietwagen, Flüge, Servicepaket, Reiseschutz</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>65183</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Mauritiusplatz 1</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n"/>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>0611 34 61 10</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="n"/>
+      <c r="L3" s="13" t="n"/>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>wiesbaden4@dertour-reisebuero.de</t>
+        </is>
+      </c>
+      <c r="N3" s="13" t="n"/>
+      <c r="O3" s="13" t="inlineStr">
+        <is>
+          <t>http://www.dertour-reisebuero.de/wiesbaden4</t>
+        </is>
+      </c>
+      <c r="P3" s="13" t="n"/>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Mo 10:00-18:00; Di 10:00-18:00; Mi 10:00-18:00; Do 10:00-18:00; Fr 10:00-18:00; Sa 10:00-14:00</t>
+        </is>
+      </c>
+      <c r="R3" s="12" t="n"/>
+      <c r="S3" s="12" t="n"/>
+      <c r="T3" s="13" t="inlineStr">
+        <is>
+          <t>463 m</t>
+        </is>
+      </c>
+      <c r="U3" s="13" t="n"/>
+      <c r="V3" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/8979c275-4c71-4305-864b-ba2f7da7de5d</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>DERTOUR Reisebüro</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
+          <t>Fernreisen, Kreuzfahrten, Rundreisen, Ferienwohnung, Mietwagen, Flüge, Servicepaket, Reiseschutz</t>
+        </is>
+      </c>
+      <c r="E4" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F4" s="15" t="inlineStr">
+        <is>
+          <t>65185</t>
+        </is>
+      </c>
+      <c r="G4" s="15" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>Friedrichstraße 34</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="n"/>
+      <c r="J4" s="15" t="inlineStr">
+        <is>
+          <t>0611 30 20 97</t>
+        </is>
+      </c>
+      <c r="K4" s="15" t="n"/>
+      <c r="L4" s="15" t="n"/>
+      <c r="M4" s="15" t="inlineStr">
+        <is>
+          <t>wiesbaden2@dertour-reisebuero.de</t>
+        </is>
+      </c>
+      <c r="N4" s="15" t="n"/>
+      <c r="O4" s="15" t="inlineStr">
+        <is>
+          <t>http://www.dertour-reisebuero.de/wiesbaden2</t>
+        </is>
+      </c>
+      <c r="P4" s="15" t="n"/>
+      <c r="Q4" s="15" t="inlineStr">
+        <is>
+          <t>Mo 10:00-18:00; Di 10:00-18:00; Mi 10:00-18:00; Do 10:00-18:00; Fr 10:00-18:00</t>
+        </is>
+      </c>
+      <c r="R4" s="14" t="n"/>
+      <c r="S4" s="14" t="n"/>
+      <c r="T4" s="15" t="inlineStr">
+        <is>
+          <t>604 m</t>
+        </is>
+      </c>
+      <c r="U4" s="15" t="n"/>
+      <c r="V4" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/d6e13499-f7d7-4201-bf30-6fed1a4817b0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Schramm Bernhard u. Maria-Luise Ferienwohnungvermietung</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungvermietung</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>65189</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Mainzer Str. 88B</t>
+        </is>
+      </c>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>0611 76 10 68</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="n"/>
+      <c r="L5" s="13" t="n"/>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>webmaster@wiesbaden-ferienwohnungen.de</t>
+        </is>
+      </c>
+      <c r="N5" s="13" t="n"/>
+      <c r="O5" s="13" t="inlineStr">
+        <is>
+          <t>https://www.wiesbaden-ferienwohnungen.de/</t>
+        </is>
+      </c>
+      <c r="P5" s="13" t="n"/>
+      <c r="Q5" s="13" t="n"/>
+      <c r="R5" s="12" t="n"/>
+      <c r="S5" s="12" t="n"/>
+      <c r="T5" s="13" t="inlineStr">
+        <is>
+          <t>1,8 km</t>
+        </is>
+      </c>
+      <c r="U5" s="13" t="n"/>
+      <c r="V5" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/6c77c1c6-fb1e-4ced-82f7-f928d06e0c47</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Doleschal Ferienwohnung</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Appartment, Ferienwohnung, Zeitmiete</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F6" s="15" t="inlineStr">
+        <is>
+          <t>65187</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Volkerstr. 47</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="n"/>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>0611 2 38 89 79</t>
+        </is>
+      </c>
+      <c r="K6" s="15" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="15" t="inlineStr">
+        <is>
+          <t>info@ferienwohnung-doleschal.de</t>
+        </is>
+      </c>
+      <c r="N6" s="15" t="n"/>
+      <c r="O6" s="15" t="inlineStr">
+        <is>
+          <t>http://www.ferienwohnung-doleschal.de/</t>
+        </is>
+      </c>
+      <c r="P6" s="15" t="n"/>
+      <c r="Q6" s="15" t="n"/>
+      <c r="R6" s="14" t="n"/>
+      <c r="S6" s="14" t="n"/>
+      <c r="T6" s="15" t="inlineStr">
+        <is>
+          <t>2,9 km</t>
+        </is>
+      </c>
+      <c r="U6" s="15" t="n"/>
+      <c r="V6" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/8c231103-c7b6-4b04-b652-32557b5c659e</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Wohnraum Becker Ferienwohnungen in Wiesbaden</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen, Appartmentvermietung</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>65199</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Helgoländer Str. 8</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>0611 4 19 01 05</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="13" t="n"/>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>info@wohnraumbecker.de</t>
+        </is>
+      </c>
+      <c r="N7" s="13" t="n"/>
+      <c r="O7" s="13" t="inlineStr">
+        <is>
+          <t>http://www.wohnraumbecker.de/</t>
+        </is>
+      </c>
+      <c r="P7" s="13" t="n"/>
+      <c r="Q7" s="13" t="n"/>
+      <c r="R7" s="12" t="n"/>
+      <c r="S7" s="12" t="n"/>
+      <c r="T7" s="13" t="inlineStr">
+        <is>
+          <t>3,6 km</t>
+        </is>
+      </c>
+      <c r="U7" s="13" t="n"/>
+      <c r="V7" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/064d40d2-8785-41d9-8794-ab619d8cf034</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Apartment Aaron-Ferienwohnung</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
+          <t>65203</t>
+        </is>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Wingertstr. 24c</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>0611 24 08 14 34</t>
+        </is>
+      </c>
+      <c r="K8" s="15" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="15" t="inlineStr">
+        <is>
+          <t>ferienwohnung.aaron@gmail.com</t>
+        </is>
+      </c>
+      <c r="N8" s="15" t="n"/>
+      <c r="O8" s="15" t="inlineStr">
+        <is>
+          <t>http://www.ferienwohnung-aaron-wiesbaden.de/</t>
+        </is>
+      </c>
+      <c r="P8" s="15" t="n"/>
+      <c r="Q8" s="15" t="n"/>
+      <c r="R8" s="14" t="n"/>
+      <c r="S8" s="14" t="n"/>
+      <c r="T8" s="15" t="inlineStr">
+        <is>
+          <t>4 km</t>
+        </is>
+      </c>
+      <c r="U8" s="15" t="n"/>
+      <c r="V8" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/02bd43c9-b59d-4d85-8f5d-7cc0627a7c13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Schmuckkästle</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>65201</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Küferstr. 12</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>0176 56 84 48 12</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="n"/>
+      <c r="L9" s="13" t="n"/>
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="13" t="n"/>
+      <c r="O9" s="13" t="n"/>
+      <c r="P9" s="13" t="n"/>
+      <c r="Q9" s="13" t="n"/>
+      <c r="R9" s="12" t="n"/>
+      <c r="S9" s="12" t="n"/>
+      <c r="T9" s="13" t="inlineStr">
+        <is>
+          <t>5,8 km</t>
+        </is>
+      </c>
+      <c r="U9" s="13" t="n"/>
+      <c r="V9" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/5127315f-8b04-4d89-ade7-40733484705e</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Schmuckkästle Vermietung von Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Ferienappartment, Weinhandlung, Riesling</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>65201</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Küferstr. 12</t>
+        </is>
+      </c>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="inlineStr">
+        <is>
+          <t>0611 58 01 88 10</t>
+        </is>
+      </c>
+      <c r="K10" s="15" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="15" t="inlineStr">
+        <is>
+          <t>info@kunsttrifftwein.de</t>
+        </is>
+      </c>
+      <c r="N10" s="15" t="n"/>
+      <c r="O10" s="15" t="inlineStr">
+        <is>
+          <t>https://www.schmuckkaestle-schierstein.de/</t>
+        </is>
+      </c>
+      <c r="P10" s="15" t="n"/>
+      <c r="Q10" s="15" t="inlineStr">
+        <is>
+          <t>Do 16:00-18:30; Fr 16:00-18:30</t>
+        </is>
+      </c>
+      <c r="R10" s="14" t="n"/>
+      <c r="S10" s="14" t="n"/>
+      <c r="T10" s="15" t="inlineStr">
+        <is>
+          <t>5,8 km</t>
+        </is>
+      </c>
+      <c r="U10" s="15" t="n"/>
+      <c r="V10" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/9cedab98-76a4-48ef-b76a-de2331cf3a7a</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Maurer Anja Vermietung von Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Apartmentvermietung</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>65207</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>Bernsteinstr. 4A</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>06127 9 86 80 56</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="n"/>
+      <c r="L11" s="13" t="n"/>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>apartments-maurer@gmx.de</t>
+        </is>
+      </c>
+      <c r="N11" s="13" t="n"/>
+      <c r="O11" s="13" t="inlineStr">
+        <is>
+          <t>http://www.apartments-maurer.de/</t>
+        </is>
+      </c>
+      <c r="P11" s="13" t="n"/>
+      <c r="Q11" s="13" t="n"/>
+      <c r="R11" s="12" t="n"/>
+      <c r="S11" s="12" t="n"/>
+      <c r="T11" s="13" t="inlineStr">
+        <is>
+          <t>6,7 km</t>
+        </is>
+      </c>
+      <c r="U11" s="13" t="n"/>
+      <c r="V11" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/b3836c61-ee83-4750-8160-da33fb64b145</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Pietscher Ferienhaus</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Ferienhaus</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>55120</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Mainz</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Hauptstr. 116</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="n"/>
+      <c r="J12" s="15" t="inlineStr">
+        <is>
+          <t>0151 16 70 50 60</t>
+        </is>
+      </c>
+      <c r="K12" s="15" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="15" t="inlineStr">
+        <is>
+          <t>ferienhaus@pietscher.de</t>
+        </is>
+      </c>
+      <c r="N12" s="15" t="n"/>
+      <c r="O12" s="15" t="inlineStr">
+        <is>
+          <t>http://www.pietscher.de/</t>
+        </is>
+      </c>
+      <c r="P12" s="15" t="n"/>
+      <c r="Q12" s="15" t="n"/>
+      <c r="R12" s="14" t="n"/>
+      <c r="S12" s="14" t="n"/>
+      <c r="T12" s="15" t="inlineStr">
+        <is>
+          <t>7 km</t>
+        </is>
+      </c>
+      <c r="U12" s="15" t="n"/>
+      <c r="V12" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/2bc78ccd-7566-4491-afdc-66b96d300786</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Herberge Hof Armada</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Fremdenzimmer, Pferdepension, Lernbauernhof</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>65201</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Hof Armada 1</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="n"/>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>0611 72 38 77 50</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="n"/>
+      <c r="L13" s="13" t="n"/>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>n.schuster@hof-armada.com</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="n"/>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>http://www.hof-armada.com/</t>
+        </is>
+      </c>
+      <c r="P13" s="13" t="n"/>
+      <c r="Q13" s="13" t="n"/>
+      <c r="R13" s="12" t="n"/>
+      <c r="S13" s="12" t="n"/>
+      <c r="T13" s="13" t="inlineStr">
+        <is>
+          <t>7,1 km</t>
+        </is>
+      </c>
+      <c r="U13" s="13" t="n"/>
+      <c r="V13" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/38b2edb5-92c4-4ea2-8743-31ef1154021f</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Aparthotel Parkallee Appartements</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Appartements, Suiten</t>
+        </is>
+      </c>
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>55257</t>
+        </is>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>Budenheim</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>Budenheimer Parkallee 9</t>
+        </is>
+      </c>
+      <c r="I14" s="15" t="n"/>
+      <c r="J14" s="15" t="inlineStr">
+        <is>
+          <t>06139 29 30 28</t>
+        </is>
+      </c>
+      <c r="K14" s="15" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="15" t="inlineStr">
+        <is>
+          <t>info@aparthotel-mainz.de</t>
+        </is>
+      </c>
+      <c r="N14" s="15" t="n"/>
+      <c r="O14" s="15" t="inlineStr">
+        <is>
+          <t>http://aparthotel-mainz.de/</t>
+        </is>
+      </c>
+      <c r="P14" s="15" t="n"/>
+      <c r="Q14" s="15" t="n"/>
+      <c r="R14" s="14" t="n"/>
+      <c r="S14" s="14" t="n"/>
+      <c r="T14" s="15" t="inlineStr">
+        <is>
+          <t>7,5 km</t>
+        </is>
+      </c>
+      <c r="U14" s="15" t="n"/>
+      <c r="V14" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/ec719e4b-84bd-47c8-a7dd-d3f579f181ac</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Maurer Apartments Maurer</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Appartements, Übernachtungen</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>65207</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>06127 9 86 80 56</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="n"/>
+      <c r="L15" s="13" t="n"/>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>info@apartments-freizeitpark.de</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="n"/>
+      <c r="O15" s="13" t="inlineStr">
+        <is>
+          <t>https://www.apartments-freizeitpark.de/</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="n"/>
+      <c r="Q15" s="13" t="n"/>
+      <c r="R15" s="12" t="n"/>
+      <c r="S15" s="12" t="n"/>
+      <c r="T15" s="13" t="n"/>
+      <c r="U15" s="13" t="n"/>
+      <c r="V15" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/52b0bfcf-05cc-437c-870b-97a20015c9be</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>FeWo Gästehäuser Irmgard u. Willi Becker Gästehaus</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>65201</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Leierweg 1</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="n"/>
+      <c r="J16" s="15" t="inlineStr">
+        <is>
+          <t>0611 9 42 77-0</t>
+        </is>
+      </c>
+      <c r="K16" s="15" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
+      <c r="P16" s="15" t="n"/>
+      <c r="Q16" s="15" t="n"/>
+      <c r="R16" s="14" t="n"/>
+      <c r="S16" s="14" t="n"/>
+      <c r="T16" s="15" t="inlineStr">
+        <is>
+          <t>5,9 km</t>
+        </is>
+      </c>
+      <c r="U16" s="15" t="n"/>
+      <c r="V16" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/f332adf6-a44d-4b47-921f-3433d908c48b</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Gästehaus Stapf</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Gästehaus, Messehotel, Hotel, Ferienwohnung, Gästezimmer, Übernachtungen, Pension, Boardinghouse, Monteurzimmer</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>65187</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Lützowstr. 4</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="n"/>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>0611 8 62 02</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="n"/>
+      <c r="L17" s="13" t="n"/>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>info@gaestehaus-stapf.de</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="n"/>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gaestehaus-stapf.de/</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="n"/>
+      <c r="Q17" s="13" t="n"/>
+      <c r="R17" s="12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S17" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="T17" s="13" t="inlineStr">
+        <is>
+          <t>3,7 km</t>
+        </is>
+      </c>
+      <c r="U17" s="13" t="n"/>
+      <c r="V17" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/5295e7c0-4b4e-4c93-8c2b-a98b8dfb6277</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Seifert Rainer TV - An- und Verkauf</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D18" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnung Wiesbaden, Unterkunft, Zimmervermietung</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>65189</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>Zweibörnstr. 13</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="n"/>
+      <c r="J18" s="15" t="inlineStr">
+        <is>
+          <t>0611 4 77 05</t>
+        </is>
+      </c>
+      <c r="K18" s="15" t="n"/>
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="inlineStr">
+        <is>
+          <t>rainerseifert13@googlemail.com</t>
+        </is>
+      </c>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="inlineStr">
+        <is>
+          <t>https://www.ferienwohnung-wiesbaden-zweibornstrasse.de/</t>
+        </is>
+      </c>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+      <c r="R18" s="14" t="n"/>
+      <c r="S18" s="14" t="n"/>
+      <c r="T18" s="15" t="inlineStr">
+        <is>
+          <t>2,7 km</t>
+        </is>
+      </c>
+      <c r="U18" s="15" t="n"/>
+      <c r="V18" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/0564ea8c-7dee-4223-ac92-e7efd8bed1d3</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Günaydin Masholtan Hotel</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Gästehaus, Dreibettzimmer, Vierbettzimmer, Übernachtung, Hotel, günstiges Hotel, Ferienwohnung, Monteurzimmer, Messezimmer, Monteurunterkunft, günstige Übernachtung, Hotel garni, M</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>65201</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>Wiesbaden</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Karl-Lehr-Str. 24</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="n"/>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>0611 2 00 20</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="n"/>
+      <c r="L19" s="13" t="n"/>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>hotel.link@t-online.de</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="n"/>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>https://www.hotellink-wiesbaden.de/</t>
+        </is>
+      </c>
+      <c r="P19" s="13" t="n"/>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Mo 07:00-22:00; Di 07:00-22:00; Mi 07:00-22:00; Do 07:00-22:00; Fr 07:00-22:00; Sa 07:00-22:00; So 07:00-22:00</t>
+        </is>
+      </c>
+      <c r="R19" s="12" t="n"/>
+      <c r="S19" s="12" t="n"/>
+      <c r="T19" s="13" t="inlineStr">
+        <is>
+          <t>5,4 km</t>
+        </is>
+      </c>
+      <c r="U19" s="13" t="n"/>
+      <c r="V19" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/4828f0e0-afd1-483a-8d3f-56e4e1c83ebf</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Reisestern Reisebüro</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Omnibus, Omnibusbetriebe, Kreuzfahrt, Reisebüro, Ferienhaus, Ferienwohnung, Fernreise, Camperreise, Last Minute Reise, Städtereise, Busreise, Strandurlaub, Schiffsreise, Wanderreis</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>65396</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>Walluf</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Erikaweg 2</t>
+        </is>
+      </c>
+      <c r="I20" s="15" t="n"/>
+      <c r="J20" s="15" t="inlineStr">
+        <is>
+          <t>06123 70 44 00</t>
+        </is>
+      </c>
+      <c r="K20" s="15" t="n"/>
+      <c r="L20" s="15" t="n"/>
+      <c r="M20" s="15" t="inlineStr">
+        <is>
+          <t>info@reisestern-walluf.de</t>
+        </is>
+      </c>
+      <c r="N20" s="15" t="n"/>
+      <c r="O20" s="15" t="inlineStr">
+        <is>
+          <t>http://www.reisebuero-reisestern.de/</t>
+        </is>
+      </c>
+      <c r="P20" s="15" t="n"/>
+      <c r="Q20" s="15" t="inlineStr">
+        <is>
+          <t>Mo 09:30-13:00; Mo 15:00-18:30; Di 09:30-13:00; Di 15:00-18:30; Mi 09:30-13:00; Do 09:30-13:00; Do 15:00-18:30; Fr 09:30-13:00; Fr 15:00-18:30; Sa 10:00-13:00</t>
+        </is>
+      </c>
+      <c r="R20" s="14" t="n"/>
+      <c r="S20" s="14" t="n"/>
+      <c r="T20" s="15" t="inlineStr">
+        <is>
+          <t>7,9 km</t>
+        </is>
+      </c>
+      <c r="U20" s="15" t="n"/>
+      <c r="V20" s="15" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/5d4fd17d-24cd-4ed1-9055-51a95fcf1904</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Apartmenthaus am Achteck</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Ferienwohnungen</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>37,7 km</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Hessen</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>64289</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="inlineStr">
+        <is>
+          <t>Darmstadt</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Mauerstr. 15</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>0179 1 22 10 30</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="13" t="n"/>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t>rene.bach@web.de</t>
+        </is>
+      </c>
+      <c r="N21" s="13" t="n"/>
+      <c r="O21" s="13" t="inlineStr">
+        <is>
+          <t>https://apartmenthaus-am-achteck.bookingturbo.com/de/</t>
+        </is>
+      </c>
+      <c r="P21" s="13" t="n"/>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Apartments, Apartmentvermietung, Ferienwohnung, Kurzzeitwohnung, Messeunterkunft, Messezimmer, Monteurswohnung, Monteurunterkunft, Zimmervermietung, Messeapartments</t>
+        </is>
+      </c>
+      <c r="R21" s="12" t="n"/>
+      <c r="S21" s="12" t="n"/>
+      <c r="T21" s="13" t="n"/>
+      <c r="U21" s="13" t="n"/>
+      <c r="V21" s="13" t="inlineStr">
+        <is>
+          <t>https://www.gelbeseiten.de/gsbiz/68a73bb6-672f-48e3-b677-2e341473fd67</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:V1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>